<commit_message>
TAREFA FORMULÁRIO 2 concluída
</commit_message>
<xml_diff>
--- a/Avancado/13 - Atingir Meta.xlsx
+++ b/Avancado/13 - Atingir Meta.xlsx
@@ -1,15 +1,21 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
-  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
-  <workbookPr defaultThemeVersion="164011"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="20730"/>
+  <workbookPr codeName="EstaPastaDeTrabalho"/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4533F92-31C5-4014-A776-FF6B93FB27CD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645"/>
+    <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Plan1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="162913"/>
+  <calcPr calcId="179021"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -18,8 +24,28 @@
 </workbook>
 </file>
 
+<file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+  <si>
+    <t>Preço Unitário</t>
+  </si>
+  <si>
+    <t>Custo variável unitário</t>
+  </si>
+  <si>
+    <t>Custo Fixo</t>
+  </si>
+  <si>
+    <t>Quantidade</t>
+  </si>
+  <si>
+    <t>Lucro</t>
+  </si>
+</sst>
+</file>
+
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" mc:Ignorable="x14ac x16r2">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
@@ -37,7 +63,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +71,37 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="1">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
+    <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -330,10 +381,66 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
-  <dimension ref="A1"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
+  <sheetPr codeName="Planilha1"/>
+  <dimension ref="A1:E5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
-  <sheetData/>
+  <cols>
+    <col min="1" max="1" width="27.42578125" customWidth="1"/>
+    <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="27.42578125" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B1" s="2">
+        <v>43.7</v>
+      </c>
+      <c r="D1" s="4"/>
+      <c r="E1" s="4"/>
+    </row>
+    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B2" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="D2" s="4"/>
+      <c r="E2" s="4"/>
+    </row>
+    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B3" s="2">
+        <v>34500</v>
+      </c>
+      <c r="D3" s="4"/>
+      <c r="E3" s="4"/>
+    </row>
+    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B4" s="3">
+        <v>1875</v>
+      </c>
+      <c r="D4" s="4"/>
+      <c r="E4" s="4"/>
+    </row>
+    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="A5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B5" s="2">
+        <f>(B1-B2)*B4</f>
+        <v>34500.000000000007</v>
+      </c>
+    </row>
+  </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
TAREFA FILTRO AVANÇADO 2 concluída
</commit_message>
<xml_diff>
--- a/Avancado/13 - Atingir Meta.xlsx
+++ b/Avancado/13 - Atingir Meta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F4533F92-31C5-4014-A776-FF6B93FB27CD}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBAEF80-94F1-43D4-9D1F-754651B0AAC7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="5" uniqueCount="5">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
   <si>
     <t>Preço Unitário</t>
   </si>
@@ -40,13 +40,35 @@
   </si>
   <si>
     <t>Lucro</t>
+  </si>
+  <si>
+    <t>Valor desejado</t>
+  </si>
+  <si>
+    <t>Prazo desejado</t>
+  </si>
+  <si>
+    <t>Prestação desejada</t>
+  </si>
+  <si>
+    <t>Taxa de juros necessária</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1" x14ac:knownFonts="1">
+  <numFmts count="1">
+    <numFmt numFmtId="44" formatCode="_-&quot;R$&quot;\ * #,##0.00_-;\-&quot;R$&quot;\ * #,##0.00_-;_-&quot;R$&quot;\ * &quot;-&quot;??_-;_-@_-"/>
+  </numFmts>
+  <fonts count="2" x14ac:knownFonts="1">
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -87,8 +109,9 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
   <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
@@ -99,11 +122,10 @@
     <xf numFmtId="1" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
+    <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
+    <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <dxfs count="0"/>
@@ -383,61 +405,108 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:E5"/>
+  <dimension ref="A1:H5"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" customWidth="1"/>
     <col min="2" max="2" width="9.28515625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="27.42578125" customWidth="1"/>
+    <col min="7" max="7" width="22.7109375" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2">
         <v>43.7</v>
       </c>
-      <c r="D1" s="4"/>
-      <c r="E1" s="4"/>
+      <c r="D1" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E1" s="2">
+        <v>43.7</v>
+      </c>
+      <c r="G1" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H1" s="4">
+        <v>8000</v>
+      </c>
     </row>
-    <row r="2" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
       <c r="B2" s="2">
         <v>25.3</v>
       </c>
-      <c r="D2" s="4"/>
-      <c r="E2" s="4"/>
+      <c r="D2" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E2" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="G2" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H2" s="1">
+        <v>24</v>
+      </c>
     </row>
-    <row r="3" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
       <c r="B3" s="2">
         <v>34500</v>
       </c>
-      <c r="D3" s="4"/>
-      <c r="E3" s="4"/>
+      <c r="D3" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E3" s="2">
+        <v>34500</v>
+      </c>
+      <c r="G3" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H3" s="4">
+        <v>400</v>
+      </c>
     </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
       <c r="B4" s="3">
         <v>1875</v>
       </c>
-      <c r="D4" s="4"/>
-      <c r="E4" s="4"/>
+      <c r="D4" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E4" s="3">
+        <v>4347.8260869565211</v>
+      </c>
+      <c r="G4" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H4" s="1"/>
     </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
       <c r="B5" s="2">
         <f>(B1-B2)*B4</f>
         <v>34500.000000000007</v>
+      </c>
+      <c r="D5" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E5" s="2">
+        <f>(E1-E2)*E4</f>
+        <v>80000</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
TAREFA 13 Atingir Meta - Parcialmente Concluída
</commit_message>
<xml_diff>
--- a/Avancado/13 - Atingir Meta.xlsx
+++ b/Avancado/13 - Atingir Meta.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{FEBAEF80-94F1-43D4-9D1F-754651B0AAC7}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126FA8F4-82B5-450D-8B96-B71B07D000B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -109,11 +109,12 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="2">
+  <cellStyleXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
+    <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="5">
+  <cellXfs count="6">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1"/>
     <xf numFmtId="2" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
@@ -123,10 +124,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="44" fontId="0" fillId="0" borderId="1" xfId="1" applyFont="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="0" borderId="1" xfId="2" applyFont="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="2">
+  <cellStyles count="3">
     <cellStyle name="Moeda" xfId="1" builtinId="4"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="2" builtinId="5"/>
   </cellStyles>
   <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
@@ -472,7 +475,8 @@
         <v>7</v>
       </c>
       <c r="H3" s="4">
-        <v>400</v>
+        <f>H1/H2*H4</f>
+        <v>400.00000000000006</v>
       </c>
     </row>
     <row r="4" spans="1:8" x14ac:dyDescent="0.25">
@@ -491,7 +495,9 @@
       <c r="G4" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="H4" s="1"/>
+      <c r="H4" s="5">
+        <v>1.2000000000000002</v>
+      </c>
     </row>
     <row r="5" spans="1:8" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">

</xml_diff>

<commit_message>
TAREFA 16 CONCLUíDA - importação de dados
</commit_message>
<xml_diff>
--- a/Avancado/13 - Atingir Meta.xlsx
+++ b/Avancado/13 - Atingir Meta.xlsx
@@ -5,10 +5,10 @@
   <workbookPr codeName="EstaPastaDeTrabalho"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-completo\Avancado\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\wilck.alunos\Desktop\EXCEL-COMPLETO\Avancado\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{126FA8F4-82B5-450D-8B96-B71B07D000B9}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{97380E0B-6796-4767-B1FC-935D3D5D035A}" xr6:coauthVersionLast="36" xr6:coauthVersionMax="36" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="0" windowWidth="22260" windowHeight="12645" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="14" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="28" uniqueCount="9">
   <si>
     <t>Preço Unitário</t>
   </si>
@@ -408,7 +408,7 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
   <sheetPr codeName="Planilha1"/>
-  <dimension ref="A1:H5"/>
+  <dimension ref="A1:J11"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="27.42578125" customWidth="1"/>
@@ -418,7 +418,7 @@
     <col min="8" max="8" width="12.140625" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="1" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -437,8 +437,11 @@
       <c r="H1" s="4">
         <v>8000</v>
       </c>
-    </row>
-    <row r="2" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J1">
+        <v>10.000000000000002</v>
+      </c>
+    </row>
+    <row r="2" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
@@ -457,8 +460,11 @@
       <c r="H2" s="1">
         <v>24</v>
       </c>
-    </row>
-    <row r="3" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J2">
+        <v>100</v>
+      </c>
+    </row>
+    <row r="3" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A3" s="1" t="s">
         <v>2</v>
       </c>
@@ -478,8 +484,12 @@
         <f>H1/H2*H4</f>
         <v>400.00000000000006</v>
       </c>
-    </row>
-    <row r="4" spans="1:8" x14ac:dyDescent="0.25">
+      <c r="J3">
+        <f>J1*J2</f>
+        <v>1000.0000000000002</v>
+      </c>
+    </row>
+    <row r="4" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
         <v>3</v>
       </c>
@@ -499,7 +509,7 @@
         <v>1.2000000000000002</v>
       </c>
     </row>
-    <row r="5" spans="1:8" x14ac:dyDescent="0.25">
+    <row r="5" spans="1:10" x14ac:dyDescent="0.25">
       <c r="A5" s="1" t="s">
         <v>4</v>
       </c>
@@ -512,6 +522,99 @@
       </c>
       <c r="E5" s="2">
         <f>(E1-E2)*E4</f>
+        <v>80000</v>
+      </c>
+    </row>
+    <row r="7" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B7" s="2">
+        <v>43.7</v>
+      </c>
+      <c r="D7" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="E7" s="2">
+        <v>43.7</v>
+      </c>
+      <c r="G7" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="H7" s="4">
+        <v>8000</v>
+      </c>
+    </row>
+    <row r="8" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="B8" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="D8" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="E8" s="2">
+        <v>25.3</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="H8" s="1">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="9" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="B9" s="2">
+        <v>34500</v>
+      </c>
+      <c r="D9" s="1" t="s">
+        <v>2</v>
+      </c>
+      <c r="E9" s="2">
+        <v>34500</v>
+      </c>
+      <c r="G9" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="H9" s="4">
+        <f>H7/H8*H10</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="B10" s="3"/>
+      <c r="D10" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="E10" s="3">
+        <v>4347.8260869565211</v>
+      </c>
+      <c r="G10" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="H10" s="5"/>
+    </row>
+    <row r="11" spans="1:10" x14ac:dyDescent="0.25">
+      <c r="A11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="B11" s="2">
+        <f>(B7-B8)*B10</f>
+        <v>0</v>
+      </c>
+      <c r="D11" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="E11" s="2">
+        <f>(E7-E8)*E10</f>
         <v>80000</v>
       </c>
     </row>

</xml_diff>